<commit_message>
Updated dimmer settings and final adjustments made.
</commit_message>
<xml_diff>
--- a/kicad/ELSONIC/POWER_BD_SV3/POWER_BD_SV2-top-pos.xlsx
+++ b/kicad/ELSONIC/POWER_BD_SV3/POWER_BD_SV2-top-pos.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_AllData\06_Embedded_Proj\KiCAD\ELSONIC\POWER_BD_SV3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{6F71C8A0-3381-49BD-B197-BD7D949103CC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B592609D-90C6-4C73-8570-2F6B93620DB9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30810" yWindow="345" windowWidth="24960" windowHeight="14205"/>
+    <workbookView xWindow="30915" yWindow="630" windowWidth="24960" windowHeight="14205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="POWER_BD_SV3-top-pos" sheetId="1" r:id="rId1"/>
@@ -157,9 +157,6 @@
     <t>R12</t>
   </si>
   <si>
-    <t>820R</t>
-  </si>
-  <si>
     <t>R13</t>
   </si>
   <si>
@@ -181,21 +178,12 @@
     <t>R17</t>
   </si>
   <si>
-    <t>68K</t>
-  </si>
-  <si>
     <t>R18</t>
   </si>
   <si>
-    <t>1K/F</t>
-  </si>
-  <si>
     <t>R19</t>
   </si>
   <si>
-    <t>40K/F</t>
-  </si>
-  <si>
     <t>R20</t>
   </si>
   <si>
@@ -221,12 +209,28 @@
   </si>
   <si>
     <t>100R</t>
+  </si>
+  <si>
+    <t>68K/F</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>820R/F</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>2K/F</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>39K/F</t>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1195,16 +1199,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9" style="1"/>
-    <col min="3" max="3" width="13.5" customWidth="1"/>
+    <col min="1" max="1" width="5.125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
     <col min="4" max="4" width="14.375" customWidth="1"/>
-    <col min="5" max="5" width="10.125" customWidth="1"/>
+    <col min="5" max="5" width="8.625" customWidth="1"/>
     <col min="6" max="6" width="9.5" customWidth="1"/>
-    <col min="7" max="8" width="10" customWidth="1"/>
+    <col min="7" max="7" width="8.5" customWidth="1"/>
+    <col min="8" max="8" width="7.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -1811,7 +1816,7 @@
         <v>44</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>33</v>
@@ -1834,10 +1839,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>47</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>33</v>
@@ -1860,10 +1865,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>33</v>
@@ -1886,10 +1891,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>33</v>
@@ -1912,10 +1917,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>33</v>
@@ -1938,10 +1943,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>33</v>
@@ -1964,10 +1969,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>33</v>
@@ -1990,10 +1995,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>33</v>
@@ -2016,10 +2021,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>33</v>
@@ -2042,7 +2047,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>32</v>
@@ -2068,10 +2073,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>33</v>
@@ -2094,10 +2099,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>33</v>
@@ -2120,10 +2125,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>33</v>

</xml_diff>